<commit_message>
Added "Sensibili" category for all macronutrients. The edit_ai_response window does not close automatically anymore after downloading.
</commit_message>
<xml_diff>
--- a/static/esempio_paziente_completo_filled.xlsx
+++ b/static/esempio_paziente_completo_filled.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio Base" sheetId="1" state="visible" r:id="rId3"/>
@@ -1017,7 +1017,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="90">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1246,10 +1246,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1372,14 +1368,6 @@
     </xf>
     <xf numFmtId="164" fontId="19" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -1726,7 +1714,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -2682,7 +2670,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="n">
         <v>31</v>
       </c>
@@ -2851,7 +2839,7 @@
       <c r="J5" s="37"/>
       <c r="K5" s="38"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E6" s="39" t="s">
         <v>9</v>
       </c>
@@ -3185,7 +3173,7 @@
         <v>40</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="G22" s="12" t="s">
         <v>59</v>
@@ -3598,8 +3586,8 @@
       <c r="M13" s="35"/>
       <c r="N13" s="36"/>
       <c r="O13" s="37"/>
-      <c r="P13" s="57"/>
-      <c r="Q13" s="57"/>
+      <c r="P13" s="4"/>
+      <c r="Q13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8"/>
@@ -3628,13 +3616,13 @@
       <c r="A15" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="57" t="s">
         <v>124</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="57" t="s">
         <v>125</v>
       </c>
-      <c r="D15" s="59" t="s">
+      <c r="D15" s="58" t="s">
         <v>35</v>
       </c>
       <c r="E15" s="22" t="s">
@@ -3661,13 +3649,13 @@
       <c r="A16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="57" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="57" t="s">
         <v>126</v>
       </c>
-      <c r="D16" s="59" t="s">
+      <c r="D16" s="58" t="s">
         <v>40</v>
       </c>
       <c r="E16" s="22" t="s">
@@ -3694,10 +3682,10 @@
       <c r="A17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="57" t="s">
         <v>128</v>
       </c>
       <c r="D17" s="22" t="s">
@@ -3727,10 +3715,10 @@
       <c r="A18" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="59" t="s">
         <v>129</v>
       </c>
       <c r="D18" s="28" t="s">
@@ -3760,10 +3748,10 @@
       <c r="A19" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="60" t="s">
         <v>112</v>
       </c>
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="60" t="s">
         <v>130</v>
       </c>
       <c r="D19" s="22" t="s">
@@ -3793,13 +3781,13 @@
       <c r="A20" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B20" s="62" t="s">
+      <c r="B20" s="61" t="s">
         <v>112</v>
       </c>
-      <c r="C20" s="62" t="s">
+      <c r="C20" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="D20" s="59" t="s">
+      <c r="D20" s="58" t="s">
         <v>36</v>
       </c>
       <c r="E20" s="22" t="s">
@@ -3826,13 +3814,13 @@
       <c r="A21" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="58" t="s">
+      <c r="B21" s="57" t="s">
         <v>132</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="57" t="s">
         <v>133</v>
       </c>
-      <c r="D21" s="59" t="s">
+      <c r="D21" s="58" t="s">
         <v>40</v>
       </c>
       <c r="E21" s="22" t="s">
@@ -3859,10 +3847,10 @@
       <c r="A22" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B22" s="58" t="s">
+      <c r="B22" s="57" t="s">
         <v>135</v>
       </c>
-      <c r="C22" s="58" t="s">
+      <c r="C22" s="57" t="s">
         <v>136</v>
       </c>
       <c r="D22" s="22" t="s">
@@ -3892,10 +3880,10 @@
       <c r="A23" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B23" s="62" t="s">
+      <c r="B23" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="62" t="s">
+      <c r="C23" s="61" t="s">
         <v>92</v>
       </c>
       <c r="D23" s="28" t="s">
@@ -3925,10 +3913,10 @@
       <c r="A24" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B24" s="58" t="s">
+      <c r="B24" s="57" t="s">
         <v>89</v>
       </c>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="57" t="s">
         <v>90</v>
       </c>
       <c r="D24" s="22" t="s">
@@ -3971,7 +3959,7 @@
       <c r="N25" s="6"/>
       <c r="O25" s="8"/>
       <c r="P25" s="8"/>
-      <c r="Q25" s="57"/>
+      <c r="Q25" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4030,25 +4018,25 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="15" style="2" width="5.01"/>
   </cols>
   <sheetData>
-    <row r="1" s="64" customFormat="true" ht="58.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="63" t="s">
+    <row r="1" s="63" customFormat="true" ht="58.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="62" t="s">
         <v>137</v>
       </c>
-      <c r="B1" s="63"/>
-      <c r="C1" s="63"/>
-      <c r="D1" s="63"/>
-      <c r="E1" s="63"/>
-      <c r="F1" s="63"/>
-      <c r="G1" s="63"/>
-      <c r="H1" s="63"/>
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
     </row>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="65" t="s">
+      <c r="A2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="65"/>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
+      <c r="B2" s="64"/>
+      <c r="C2" s="64"/>
+      <c r="D2" s="64"/>
       <c r="E2" s="9"/>
       <c r="F2" s="10" t="s">
         <v>2</v>
@@ -4118,7 +4106,7 @@
       <c r="I5" s="36"/>
       <c r="J5" s="37"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -4266,10 +4254,10 @@
       <c r="A15" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="57" t="s">
         <v>138</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="57" t="s">
         <v>139</v>
       </c>
       <c r="D15" s="22" t="s">
@@ -4290,10 +4278,10 @@
       <c r="A16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="57" t="s">
         <v>140</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="57" t="s">
         <v>141</v>
       </c>
       <c r="D16" s="28" t="s">
@@ -4314,10 +4302,10 @@
       <c r="A17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="57" t="s">
         <v>143</v>
       </c>
       <c r="D17" s="28" t="s">
@@ -4338,10 +4326,10 @@
       <c r="A18" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="57" t="s">
         <v>144</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="59" t="s">
         <v>145</v>
       </c>
       <c r="D18" s="22" t="s">
@@ -4362,10 +4350,10 @@
       <c r="A19" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="C19" s="58" t="s">
+      <c r="C19" s="57" t="s">
         <v>147</v>
       </c>
       <c r="D19" s="28" t="s">
@@ -4386,10 +4374,10 @@
       <c r="A20" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B20" s="58" t="s">
+      <c r="B20" s="57" t="s">
         <v>148</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="57" t="s">
         <v>149</v>
       </c>
       <c r="D20" s="22" t="s">
@@ -4410,10 +4398,10 @@
       <c r="A21" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="60" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="60" t="s">
         <v>151</v>
       </c>
       <c r="D21" s="28" t="s">
@@ -4434,10 +4422,10 @@
       <c r="A22" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B22" s="62" t="s">
+      <c r="B22" s="61" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="62" t="s">
+      <c r="C22" s="61" t="s">
         <v>153</v>
       </c>
       <c r="D22" s="22" t="s">
@@ -4458,10 +4446,10 @@
       <c r="A23" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="57" t="s">
         <v>154</v>
       </c>
-      <c r="C23" s="58" t="s">
+      <c r="C23" s="57" t="s">
         <v>155</v>
       </c>
       <c r="D23" s="22" t="s">
@@ -4482,10 +4470,10 @@
       <c r="A24" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B24" s="58" t="s">
+      <c r="B24" s="57" t="s">
         <v>154</v>
       </c>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="57" t="s">
         <v>156</v>
       </c>
       <c r="D24" s="22" t="s">
@@ -4506,10 +4494,10 @@
       <c r="A25" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="57" t="s">
         <v>157</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="57" t="s">
         <v>158</v>
       </c>
       <c r="D25" s="22" t="s">
@@ -4530,10 +4518,10 @@
       <c r="A26" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B26" s="58" t="s">
+      <c r="B26" s="57" t="s">
         <v>160</v>
       </c>
-      <c r="C26" s="58" t="s">
+      <c r="C26" s="57" t="s">
         <v>161</v>
       </c>
       <c r="D26" s="22" t="s">
@@ -4554,10 +4542,10 @@
       <c r="A27" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B27" s="58" t="s">
+      <c r="B27" s="57" t="s">
         <v>160</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="57" t="s">
         <v>162</v>
       </c>
       <c r="D27" s="22" t="s">
@@ -4578,10 +4566,10 @@
       <c r="A28" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B28" s="58" t="s">
+      <c r="B28" s="57" t="s">
         <v>163</v>
       </c>
-      <c r="C28" s="58" t="s">
+      <c r="C28" s="57" t="s">
         <v>164</v>
       </c>
       <c r="D28" s="22" t="s">
@@ -4602,10 +4590,10 @@
       <c r="A29" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="57" t="s">
         <v>163</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="57" t="s">
         <v>165</v>
       </c>
       <c r="D29" s="28" t="s">
@@ -4626,10 +4614,10 @@
       <c r="A30" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B30" s="58" t="s">
+      <c r="B30" s="57" t="s">
         <v>163</v>
       </c>
-      <c r="C30" s="58" t="s">
+      <c r="C30" s="57" t="s">
         <v>166</v>
       </c>
       <c r="D30" s="28" t="s">
@@ -4647,106 +4635,106 @@
       <c r="J30" s="37"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="66"/>
-      <c r="B31" s="67"/>
-      <c r="C31" s="67"/>
-      <c r="D31" s="68"/>
-      <c r="E31" s="68"/>
-      <c r="F31" s="69"/>
+      <c r="A31" s="65"/>
+      <c r="B31" s="66"/>
+      <c r="C31" s="66"/>
+      <c r="D31" s="67"/>
+      <c r="E31" s="67"/>
+      <c r="F31" s="68"/>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
       <c r="J31" s="7"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="66"/>
-      <c r="B32" s="70"/>
-      <c r="C32" s="71"/>
-      <c r="D32" s="68"/>
-      <c r="E32" s="68"/>
-      <c r="F32" s="69"/>
+      <c r="A32" s="65"/>
+      <c r="B32" s="69"/>
+      <c r="C32" s="70"/>
+      <c r="D32" s="67"/>
+      <c r="E32" s="67"/>
+      <c r="F32" s="68"/>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
       <c r="I32" s="7"/>
       <c r="J32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="66"/>
-      <c r="B33" s="70"/>
-      <c r="C33" s="70"/>
-      <c r="D33" s="68"/>
-      <c r="E33" s="68"/>
-      <c r="F33" s="69"/>
+      <c r="A33" s="65"/>
+      <c r="B33" s="69"/>
+      <c r="C33" s="69"/>
+      <c r="D33" s="67"/>
+      <c r="E33" s="67"/>
+      <c r="F33" s="68"/>
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
       <c r="I33" s="7"/>
       <c r="J33" s="7"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="66"/>
-      <c r="B34" s="70"/>
-      <c r="C34" s="70"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="68"/>
-      <c r="F34" s="69"/>
+      <c r="A34" s="65"/>
+      <c r="B34" s="69"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="67"/>
+      <c r="E34" s="67"/>
+      <c r="F34" s="68"/>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="7"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="66"/>
-      <c r="B35" s="70"/>
-      <c r="C35" s="70"/>
-      <c r="D35" s="68"/>
-      <c r="E35" s="68"/>
-      <c r="F35" s="69"/>
+      <c r="A35" s="65"/>
+      <c r="B35" s="69"/>
+      <c r="C35" s="69"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
+      <c r="F35" s="68"/>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="7"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="66"/>
-      <c r="B36" s="72"/>
-      <c r="C36" s="73"/>
-      <c r="D36" s="74"/>
-      <c r="E36" s="75"/>
-      <c r="F36" s="69"/>
+      <c r="A36" s="65"/>
+      <c r="B36" s="71"/>
+      <c r="C36" s="72"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="74"/>
+      <c r="F36" s="68"/>
       <c r="G36" s="7"/>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="7"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="66"/>
-      <c r="B37" s="72"/>
-      <c r="C37" s="73"/>
-      <c r="D37" s="74"/>
-      <c r="E37" s="75"/>
-      <c r="F37" s="69"/>
+      <c r="A37" s="65"/>
+      <c r="B37" s="71"/>
+      <c r="C37" s="72"/>
+      <c r="D37" s="73"/>
+      <c r="E37" s="74"/>
+      <c r="F37" s="68"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="7"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="72"/>
-      <c r="C38" s="73"/>
-      <c r="D38" s="75"/>
-      <c r="E38" s="75"/>
-      <c r="F38" s="69"/>
+      <c r="B38" s="71"/>
+      <c r="C38" s="72"/>
+      <c r="D38" s="74"/>
+      <c r="E38" s="74"/>
+      <c r="F38" s="68"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7"/>
       <c r="I38" s="7"/>
       <c r="J38" s="7"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="72"/>
-      <c r="C39" s="73"/>
-      <c r="D39" s="75"/>
-      <c r="E39" s="75"/>
-      <c r="F39" s="69"/>
+      <c r="B39" s="71"/>
+      <c r="C39" s="72"/>
+      <c r="D39" s="74"/>
+      <c r="E39" s="74"/>
+      <c r="F39" s="68"/>
       <c r="G39" s="7"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7"/>
@@ -4804,16 +4792,16 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="76" t="s">
+      <c r="A1" s="75" t="s">
         <v>167</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
@@ -4824,7 +4812,7 @@
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
-      <c r="E2" s="77"/>
+      <c r="E2" s="76"/>
       <c r="F2" s="10" t="s">
         <v>2</v>
       </c>
@@ -4893,7 +4881,7 @@
       <c r="I5" s="36"/>
       <c r="J5" s="37"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5001,7 +4989,7 @@
         <v>26</v>
       </c>
       <c r="G12" s="56"/>
-      <c r="H12" s="78"/>
+      <c r="H12" s="77"/>
       <c r="I12" s="41"/>
       <c r="J12" s="42"/>
     </row>
@@ -5041,13 +5029,13 @@
       <c r="A15" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="58" t="s">
+      <c r="B15" s="57" t="s">
         <v>168</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="57" t="s">
         <v>169</v>
       </c>
-      <c r="D15" s="79" t="s">
+      <c r="D15" s="78" t="s">
         <v>36</v>
       </c>
       <c r="E15" s="28" t="s">
@@ -5065,13 +5053,13 @@
       <c r="A16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="58" t="s">
+      <c r="B16" s="57" t="s">
         <v>170</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="57" t="s">
         <v>171</v>
       </c>
-      <c r="D16" s="79" t="s">
+      <c r="D16" s="78" t="s">
         <v>45</v>
       </c>
       <c r="E16" s="28" t="s">
@@ -5089,13 +5077,13 @@
       <c r="A17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="57" t="s">
         <v>170</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="57" t="s">
         <v>172</v>
       </c>
-      <c r="D17" s="80" t="s">
+      <c r="D17" s="79" t="s">
         <v>40</v>
       </c>
       <c r="E17" s="22" t="s">
@@ -5113,13 +5101,13 @@
       <c r="A18" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="58" t="s">
+      <c r="B18" s="57" t="s">
         <v>173</v>
       </c>
-      <c r="C18" s="60" t="s">
+      <c r="C18" s="59" t="s">
         <v>174</v>
       </c>
-      <c r="D18" s="79" t="s">
+      <c r="D18" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E18" s="28" t="s">
@@ -5137,13 +5125,13 @@
       <c r="A19" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="C19" s="58" t="s">
+      <c r="C19" s="57" t="s">
         <v>176</v>
       </c>
-      <c r="D19" s="79" t="s">
+      <c r="D19" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E19" s="28" t="s">
@@ -5161,13 +5149,13 @@
       <c r="A20" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B20" s="58" t="s">
+      <c r="B20" s="57" t="s">
         <v>177</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="57" t="s">
         <v>178</v>
       </c>
-      <c r="D20" s="79" t="s">
+      <c r="D20" s="78" t="s">
         <v>45</v>
       </c>
       <c r="E20" s="28" t="s">
@@ -5185,13 +5173,13 @@
       <c r="A21" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="61" t="s">
+      <c r="B21" s="60" t="s">
         <v>170</v>
       </c>
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="60" t="s">
         <v>179</v>
       </c>
-      <c r="D21" s="79" t="s">
+      <c r="D21" s="78" t="s">
         <v>36</v>
       </c>
       <c r="E21" s="28" t="s">
@@ -5209,13 +5197,13 @@
       <c r="A22" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B22" s="62" t="s">
+      <c r="B22" s="61" t="s">
         <v>175</v>
       </c>
-      <c r="C22" s="62" t="s">
+      <c r="C22" s="61" t="s">
         <v>180</v>
       </c>
-      <c r="D22" s="79" t="s">
+      <c r="D22" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E22" s="28" t="s">
@@ -5233,13 +5221,13 @@
       <c r="A23" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B23" s="58" t="s">
+      <c r="B23" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="C23" s="58" t="s">
+      <c r="C23" s="57" t="s">
         <v>181</v>
       </c>
-      <c r="D23" s="79" t="s">
+      <c r="D23" s="78" t="s">
         <v>36</v>
       </c>
       <c r="E23" s="28" t="s">
@@ -5257,13 +5245,13 @@
       <c r="A24" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B24" s="58" t="s">
+      <c r="B24" s="57" t="s">
         <v>175</v>
       </c>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="57" t="s">
         <v>182</v>
       </c>
-      <c r="D24" s="79" t="s">
+      <c r="D24" s="78" t="s">
         <v>36</v>
       </c>
       <c r="E24" s="28" t="s">
@@ -5281,13 +5269,13 @@
       <c r="A25" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="57" t="s">
         <v>183</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="57" t="s">
         <v>184</v>
       </c>
-      <c r="D25" s="79" t="s">
+      <c r="D25" s="78" t="s">
         <v>36</v>
       </c>
       <c r="E25" s="28" t="s">
@@ -5305,13 +5293,13 @@
       <c r="A26" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B26" s="58" t="s">
+      <c r="B26" s="57" t="s">
         <v>185</v>
       </c>
-      <c r="C26" s="58" t="s">
+      <c r="C26" s="57" t="s">
         <v>186</v>
       </c>
-      <c r="D26" s="79" t="s">
+      <c r="D26" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E26" s="28" t="s">
@@ -5329,13 +5317,13 @@
       <c r="A27" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B27" s="58" t="s">
+      <c r="B27" s="57" t="s">
         <v>187</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="57" t="s">
         <v>188</v>
       </c>
-      <c r="D27" s="79" t="s">
+      <c r="D27" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E27" s="28" t="s">
@@ -5353,13 +5341,13 @@
       <c r="A28" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B28" s="58" t="s">
+      <c r="B28" s="57" t="s">
         <v>187</v>
       </c>
-      <c r="C28" s="58" t="s">
+      <c r="C28" s="57" t="s">
         <v>189</v>
       </c>
-      <c r="D28" s="79" t="s">
+      <c r="D28" s="78" t="s">
         <v>40</v>
       </c>
       <c r="E28" s="28" t="s">
@@ -5377,13 +5365,13 @@
       <c r="A29" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B29" s="58" t="s">
+      <c r="B29" s="57" t="s">
         <v>190</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="57" t="s">
         <v>191</v>
       </c>
-      <c r="D29" s="79" t="s">
+      <c r="D29" s="78" t="s">
         <v>36</v>
       </c>
       <c r="E29" s="28" t="s">
@@ -5438,7 +5426,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="20.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="7.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="15.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="20.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="20.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="13.43"/>
@@ -5539,7 +5527,7 @@
       <c r="I5" s="36"/>
       <c r="J5" s="37"/>
     </row>
-    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5687,16 +5675,16 @@
       <c r="A15" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="81" t="s">
+      <c r="B15" s="80" t="s">
         <v>194</v>
       </c>
-      <c r="C15" s="81" t="s">
+      <c r="C15" s="80" t="s">
         <v>195</v>
       </c>
       <c r="D15" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="59" t="s">
+      <c r="E15" s="58" t="s">
         <v>35</v>
       </c>
       <c r="F15" s="12" t="s">
@@ -5711,16 +5699,16 @@
       <c r="A16" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="81" t="s">
+      <c r="B16" s="80" t="s">
         <v>194</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="80" t="s">
         <v>196</v>
       </c>
       <c r="D16" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="59" t="s">
+      <c r="E16" s="58" t="s">
         <v>40</v>
       </c>
       <c r="F16" s="12" t="s">
@@ -5735,16 +5723,16 @@
       <c r="A17" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="81" t="s">
+      <c r="B17" s="80" t="s">
         <v>197</v>
       </c>
-      <c r="C17" s="81" t="s">
+      <c r="C17" s="80" t="s">
         <v>198</v>
       </c>
-      <c r="D17" s="59" t="s">
+      <c r="D17" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="E17" s="82" t="s">
+      <c r="E17" s="81" t="s">
         <v>36</v>
       </c>
       <c r="F17" s="12" t="s">
@@ -5759,16 +5747,16 @@
       <c r="A18" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="81" t="s">
+      <c r="B18" s="80" t="s">
         <v>197</v>
       </c>
-      <c r="C18" s="81" t="s">
+      <c r="C18" s="80" t="s">
         <v>199</v>
       </c>
       <c r="D18" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="59" t="s">
+      <c r="E18" s="58" t="s">
         <v>40</v>
       </c>
       <c r="F18" s="12" t="s">
@@ -5783,16 +5771,16 @@
       <c r="A19" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B19" s="81" t="s">
+      <c r="B19" s="80" t="s">
         <v>200</v>
       </c>
-      <c r="C19" s="81" t="s">
+      <c r="C19" s="80" t="s">
         <v>201</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="82" t="s">
+      <c r="E19" s="81" t="s">
         <v>40</v>
       </c>
       <c r="F19" s="12" t="s">
@@ -5807,16 +5795,16 @@
       <c r="A20" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B20" s="81" t="s">
+      <c r="B20" s="80" t="s">
         <v>200</v>
       </c>
-      <c r="C20" s="81" t="s">
+      <c r="C20" s="80" t="s">
         <v>203</v>
       </c>
-      <c r="D20" s="59" t="s">
+      <c r="D20" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="82" t="s">
+      <c r="E20" s="81" t="s">
         <v>35</v>
       </c>
       <c r="F20" s="12" t="s">
@@ -5831,16 +5819,16 @@
       <c r="A21" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B21" s="81" t="s">
+      <c r="B21" s="80" t="s">
         <v>200</v>
       </c>
-      <c r="C21" s="81" t="s">
+      <c r="C21" s="80" t="s">
         <v>204</v>
       </c>
-      <c r="D21" s="59" t="s">
+      <c r="D21" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="E21" s="82" t="s">
+      <c r="E21" s="81" t="s">
         <v>45</v>
       </c>
       <c r="F21" s="12" t="s">
@@ -5855,16 +5843,16 @@
       <c r="A22" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B22" s="81" t="s">
+      <c r="B22" s="80" t="s">
         <v>205</v>
       </c>
-      <c r="C22" s="81" t="s">
+      <c r="C22" s="80" t="s">
         <v>206</v>
       </c>
-      <c r="D22" s="59" t="s">
+      <c r="D22" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="82" t="s">
+      <c r="E22" s="81" t="s">
         <v>36</v>
       </c>
       <c r="F22" s="12" t="s">
@@ -5879,16 +5867,16 @@
       <c r="A23" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B23" s="81" t="s">
+      <c r="B23" s="80" t="s">
         <v>207</v>
       </c>
-      <c r="C23" s="81" t="s">
+      <c r="C23" s="80" t="s">
         <v>208</v>
       </c>
-      <c r="D23" s="59" t="s">
+      <c r="D23" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="E23" s="82" t="s">
+      <c r="E23" s="81" t="s">
         <v>40</v>
       </c>
       <c r="F23" s="12" t="s">
@@ -5903,16 +5891,16 @@
       <c r="A24" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B24" s="81" t="s">
+      <c r="B24" s="80" t="s">
         <v>207</v>
       </c>
-      <c r="C24" s="81" t="s">
+      <c r="C24" s="80" t="s">
         <v>209</v>
       </c>
       <c r="D24" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="59" t="s">
+      <c r="E24" s="58" t="s">
         <v>35</v>
       </c>
       <c r="F24" s="12" t="s">
@@ -5927,16 +5915,16 @@
       <c r="A25" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B25" s="81" t="s">
+      <c r="B25" s="80" t="s">
         <v>197</v>
       </c>
-      <c r="C25" s="81" t="s">
+      <c r="C25" s="80" t="s">
         <v>210</v>
       </c>
-      <c r="D25" s="59" t="s">
+      <c r="D25" s="58" t="s">
         <v>45</v>
       </c>
-      <c r="E25" s="82" t="s">
+      <c r="E25" s="81" t="s">
         <v>40</v>
       </c>
       <c r="F25" s="12" t="s">
@@ -5951,16 +5939,16 @@
       <c r="A26" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="B26" s="81" t="s">
+      <c r="B26" s="80" t="s">
         <v>197</v>
       </c>
-      <c r="C26" s="81" t="s">
+      <c r="C26" s="80" t="s">
         <v>211</v>
       </c>
-      <c r="D26" s="59" t="s">
+      <c r="D26" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="E26" s="82" t="s">
+      <c r="E26" s="81" t="s">
         <v>36</v>
       </c>
       <c r="F26" s="12" t="s">
@@ -5975,16 +5963,16 @@
       <c r="A27" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="80" t="s">
         <v>212</v>
       </c>
-      <c r="C27" s="81" t="s">
+      <c r="C27" s="80" t="s">
         <v>213</v>
       </c>
-      <c r="D27" s="82" t="s">
+      <c r="D27" s="81" t="s">
         <v>40</v>
       </c>
-      <c r="E27" s="59" t="s">
+      <c r="E27" s="58" t="s">
         <v>45</v>
       </c>
       <c r="F27" s="12" t="s">
@@ -5999,16 +5987,16 @@
       <c r="A28" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="B28" s="81" t="s">
+      <c r="B28" s="80" t="s">
         <v>214</v>
       </c>
-      <c r="C28" s="81" t="s">
+      <c r="C28" s="80" t="s">
         <v>215</v>
       </c>
       <c r="D28" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="59" t="s">
+      <c r="E28" s="58" t="s">
         <v>35</v>
       </c>
       <c r="F28" s="12" t="s">
@@ -6023,13 +6011,13 @@
       <c r="A29" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="B29" s="81" t="s">
+      <c r="B29" s="80" t="s">
         <v>216</v>
       </c>
-      <c r="C29" s="81" t="s">
+      <c r="C29" s="80" t="s">
         <v>217</v>
       </c>
-      <c r="D29" s="59" t="s">
+      <c r="D29" s="58" t="s">
         <v>35</v>
       </c>
       <c r="E29" s="22" t="s">
@@ -6047,16 +6035,16 @@
       <c r="A30" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="B30" s="81" t="s">
+      <c r="B30" s="80" t="s">
         <v>218</v>
       </c>
-      <c r="C30" s="81" t="s">
+      <c r="C30" s="80" t="s">
         <v>219</v>
       </c>
       <c r="D30" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E30" s="59" t="s">
+      <c r="E30" s="58" t="s">
         <v>45</v>
       </c>
       <c r="F30" s="12" t="s">
@@ -6071,13 +6059,13 @@
       <c r="A31" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="B31" s="81" t="s">
+      <c r="B31" s="80" t="s">
         <v>218</v>
       </c>
-      <c r="C31" s="81" t="s">
+      <c r="C31" s="80" t="s">
         <v>220</v>
       </c>
-      <c r="D31" s="59" t="s">
+      <c r="D31" s="58" t="s">
         <v>45</v>
       </c>
       <c r="E31" s="22" t="s">
@@ -6093,10 +6081,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="8"/>
-      <c r="B32" s="58"/>
-      <c r="C32" s="83"/>
-      <c r="D32" s="80"/>
-      <c r="E32" s="79"/>
+      <c r="B32" s="57"/>
+      <c r="C32" s="82"/>
+      <c r="D32" s="79"/>
+      <c r="E32" s="78"/>
       <c r="F32" s="12"/>
       <c r="G32" s="54"/>
       <c r="H32" s="19"/>
@@ -6105,10 +6093,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="8"/>
-      <c r="B33" s="58"/>
-      <c r="C33" s="58"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="79"/>
+      <c r="B33" s="57"/>
+      <c r="C33" s="57"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="78"/>
       <c r="F33" s="12"/>
       <c r="G33" s="54"/>
       <c r="H33" s="19"/>
@@ -6117,10 +6105,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8"/>
-      <c r="B34" s="58"/>
-      <c r="C34" s="58"/>
-      <c r="D34" s="80"/>
-      <c r="E34" s="79"/>
+      <c r="B34" s="57"/>
+      <c r="C34" s="57"/>
+      <c r="D34" s="79"/>
+      <c r="E34" s="78"/>
       <c r="F34" s="12"/>
       <c r="G34" s="54"/>
       <c r="H34" s="19"/>
@@ -6129,10 +6117,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8"/>
-      <c r="B35" s="58"/>
-      <c r="C35" s="58"/>
-      <c r="D35" s="80"/>
-      <c r="E35" s="79"/>
+      <c r="B35" s="57"/>
+      <c r="C35" s="57"/>
+      <c r="D35" s="79"/>
+      <c r="E35" s="78"/>
       <c r="F35" s="12"/>
       <c r="G35" s="54"/>
       <c r="H35" s="19"/>
@@ -6141,10 +6129,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8"/>
-      <c r="B36" s="84"/>
-      <c r="C36" s="85"/>
-      <c r="D36" s="86"/>
-      <c r="E36" s="87"/>
+      <c r="B36" s="83"/>
+      <c r="C36" s="84"/>
+      <c r="D36" s="85"/>
+      <c r="E36" s="86"/>
       <c r="F36" s="12"/>
       <c r="G36" s="54"/>
       <c r="H36" s="19"/>
@@ -6153,10 +6141,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8"/>
-      <c r="B37" s="84"/>
-      <c r="C37" s="85"/>
-      <c r="D37" s="86"/>
-      <c r="E37" s="87"/>
+      <c r="B37" s="83"/>
+      <c r="C37" s="84"/>
+      <c r="D37" s="85"/>
+      <c r="E37" s="86"/>
       <c r="F37" s="12"/>
       <c r="G37" s="54"/>
       <c r="H37" s="19"/>
@@ -6165,10 +6153,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="8"/>
-      <c r="B38" s="84"/>
-      <c r="C38" s="85"/>
-      <c r="D38" s="88"/>
-      <c r="E38" s="87"/>
+      <c r="B38" s="83"/>
+      <c r="C38" s="84"/>
+      <c r="D38" s="87"/>
+      <c r="E38" s="86"/>
       <c r="F38" s="12"/>
       <c r="G38" s="54"/>
       <c r="H38" s="19"/>
@@ -6177,10 +6165,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8"/>
-      <c r="B39" s="84"/>
-      <c r="C39" s="85"/>
-      <c r="D39" s="88"/>
-      <c r="E39" s="87"/>
+      <c r="B39" s="83"/>
+      <c r="C39" s="84"/>
+      <c r="D39" s="87"/>
+      <c r="E39" s="86"/>
       <c r="F39" s="12"/>
       <c r="G39" s="54"/>
       <c r="H39" s="19"/>
@@ -6220,10 +6208,10 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="89" width="17.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="51" width="17.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="36.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="33.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="23.48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6236,7 +6224,7 @@
       <c r="E1" s="3"/>
       <c r="F1" s="3"/>
       <c r="G1" s="4"/>
-      <c r="H1" s="57"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
@@ -6245,7 +6233,7 @@
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
-      <c r="E2" s="90"/>
+      <c r="E2" s="53"/>
       <c r="F2" s="6" t="s">
         <v>2</v>
       </c>
@@ -6254,7 +6242,7 @@
     </row>
     <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8"/>
-      <c r="B3" s="57"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="10" t="s">
@@ -6272,7 +6260,7 @@
     </row>
     <row r="4" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8"/>
-      <c r="B4" s="57"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="10" t="s">
@@ -6290,9 +6278,9 @@
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8"/>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
       <c r="E5" s="10" t="s">
         <v>5</v>
       </c>
@@ -6306,11 +6294,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="16.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
-      <c r="B6" s="57"/>
-      <c r="C6" s="57"/>
-      <c r="D6" s="57"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
       <c r="E6" s="13" t="s">
         <v>9</v>
       </c>
@@ -6326,9 +6314,9 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8"/>
-      <c r="B7" s="57"/>
-      <c r="C7" s="57"/>
-      <c r="D7" s="57"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
       <c r="E7" s="13" t="s">
         <v>13</v>
       </c>
@@ -6344,9 +6332,9 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8"/>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
       <c r="E8" s="10" t="s">
         <v>17</v>
       </c>
@@ -6362,9 +6350,9 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8"/>
-      <c r="B9" s="57"/>
-      <c r="C9" s="57"/>
-      <c r="D9" s="57"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
       <c r="E9" s="10" t="s">
         <v>18</v>
       </c>
@@ -6380,9 +6368,9 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="57"/>
-      <c r="D10" s="57"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
       <c r="E10" s="10" t="s">
         <v>19</v>
       </c>
@@ -6398,9 +6386,9 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8"/>
-      <c r="B11" s="57"/>
-      <c r="C11" s="57"/>
-      <c r="D11" s="57"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
       <c r="E11" s="10" t="s">
         <v>22</v>
       </c>
@@ -6416,9 +6404,9 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8"/>
-      <c r="B12" s="57"/>
-      <c r="C12" s="57"/>
-      <c r="D12" s="57"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
         <v>24</v>
       </c>
@@ -6434,9 +6422,9 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="57"/>
-      <c r="D13" s="57"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
       <c r="E13" s="10" t="s">
         <v>28</v>
       </c>
@@ -6451,20 +6439,20 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="51.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="57"/>
-      <c r="B14" s="57"/>
-      <c r="C14" s="57"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="91" t="s">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="88" t="s">
         <v>223</v>
       </c>
-      <c r="F14" s="92" t="s">
+      <c r="F14" s="89" t="s">
         <v>224</v>
       </c>
-      <c r="G14" s="92" t="s">
+      <c r="G14" s="89" t="s">
         <v>225</v>
       </c>
-      <c r="H14" s="92"/>
+      <c r="H14" s="89"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
JSON is directly sent to the app backend
</commit_message>
<xml_diff>
--- a/static/esempio_paziente_completo_filled.xlsx
+++ b/static/esempio_paziente_completo_filled.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio Base" sheetId="1" state="visible" r:id="rId3"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="229">
   <si>
     <t xml:space="preserve">FOGLIO LAVORO GENEFOOD BASE</t>
   </si>
@@ -53,652 +53,661 @@
     <t xml:space="preserve">PAZIENTE</t>
   </si>
   <si>
+    <t xml:space="preserve">ROSSI MIRKO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verdini Giulio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mammaesempio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rossi@bla.it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">verdi@bla.it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mamma@blah.it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CODICE_FISCALE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSSKUI99E43G577V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VRDKLN46H10D891M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMESNH46D11E648G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PESO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALTEZZA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SESSO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIMITAZIONI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATA_NASCITA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11/10/1970</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/06/1989</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05/03/1988</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMMITTENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genessere</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altamedica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">predisponente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADIPOq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs17300539</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADRB1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1801253</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APOA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs5082</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APOA5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs662799</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APOE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs429358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs7412</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BDNF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs6265</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CETP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs3764261</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs708272</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FABP2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1799883</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FADS1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs174546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FADS2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs174601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1121980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1421085</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1558902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs8050136</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs9939609</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1799884</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GCKR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs780094</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GNPDA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs10938397</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs11208659</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leptin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs7799039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MC4R </t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs17700144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MC4R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs17782313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTHFR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1801131</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1801133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MTNR1B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs10830963</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PPARG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1801282</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLC30A8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs13266634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TCFL2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs7903146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMEM18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs6548238</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD PLUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALDH2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs671</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALDOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs76917243</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1800546</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLDN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs9290927</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs893051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs17501010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CYP1A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs762551</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LCT (MCM6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4988235</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HLA_DQA1-B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xxx1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQ8/DQ7.5/DQ2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DQ8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD VITA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verdi Giulio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HFE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1799945</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1800562</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMPRSS6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs855791</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4820268</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs7041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1155563</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHCR7/NADSYN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs12785878</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FUT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs602662</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOGLIOLAVORO GENEFOOD SPORT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL27A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs946053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL12A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs970547</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL5A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs12722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL1A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1800012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESR1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs2234693</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDF5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs143383</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LRP5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs3736228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1049434</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMP3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs591058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs679620</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTN3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1815739</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs2070744</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1799983</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1330363</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs2104772</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs13321</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD AGEING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL1B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs16944</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1143634</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IL6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1800796</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOD3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1799895</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPX1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1050450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1143633</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs2536512</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs13306703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs699473</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1001179</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NQO1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1800566</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOD2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4880</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1141718</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQUAPORIN3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs17553719</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD MAMMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GESTAZIONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALPL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4654748</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1256335</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs11568020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs5050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLCNKA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs848307 1a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1739843 3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1010069 4a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADD1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4961 (Gly460Trp)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEDD4L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4149601</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs2288774</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs699 (M235T)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs5051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs1532423</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PPCDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs2120019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NBDY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs4826508</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLC30A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs35623192</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rs35235055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD CONDIZIONI</t>
+  </si>
+  <si>
     <t xml:space="preserve">ROSSI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verdi Giulio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mammaesempio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rossi@bla.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">verdi@bla.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mamma@blah.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CODICE_FISCALE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSSKUI99E43G577V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VRDKLN46H10D891M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMESNH46D11E648G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PESO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALTEZZA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SESSO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13/2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIMITAZIONI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATA_NASCITA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11/10/1970</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09/06/1989</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05/03/1988</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMMITTENTE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Genessere</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altamedica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">predisponente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADIPOq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs17300539</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADRB1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1801253</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APOA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs5082</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APOA5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs662799</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APOE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs429358</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs7412</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BDNF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs6265</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CETP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs3764261</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs708272</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FABP2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1799883</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FADS1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs174546</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FADS2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs174601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1121980</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1421085</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1558902</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs8050136</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs9939609</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GCK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1799884</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GCKR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs780094</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GNPDA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs10938397</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEPR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs11208659</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leptin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs7799039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MC4R </t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs17700144</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MC4R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs17782313</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MTHFR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1801131</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1801133</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MTNR1B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs10830963</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PPARG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1801282</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLC30A8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs13266634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TCFL2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs7903146</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TMEM18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs6548238</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD PLUS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALDH2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs671</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALDOB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs76917243</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1800546</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLDN1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs9290927</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs893051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs17501010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CYP1A2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs762551</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LCT (MCM6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4988235</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HLA_DQA1-B1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">xxx1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Normale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DQ8/DQ7.5/DQ2.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DQ8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD VITA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HFE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1799945</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1800562</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TMPRSS6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs855791</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4820268</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs7041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1155563</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DHCR7/NADSYN1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs12785878</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FUT2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs602662</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOGLIOLAVORO GENEFOOD SPORT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL27A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs946053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL12A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs970547</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL5A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs12722</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL1A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1800012</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESR1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs2234693</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GDF5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs143383</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LRP5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs3736228</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MCT1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1049434</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMP3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs591058</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs679620</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1815739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOS3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs2070744</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1799983</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TNC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1330363</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs2104772</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs13321</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD AGEING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CRP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1205</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IL1B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs16944</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1143634</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IL6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1800796</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOD3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1799895</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GPX1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1050450</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1143633</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs2536512</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs13306703</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs699473</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1001179</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NQO1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1800566</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOD2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4880</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1141718</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AQUAPORIN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs17553719</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD MAMMA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GESTAZIONE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALPL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4654748</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1256335</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs11568020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs5050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CLCNKA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs848307 1a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1739843 3a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1010069 4a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADD1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4961 (Gly460Trp)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NEDD4L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4149601</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs2288774</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs699 (M235T)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs5051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs1532423</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PPCDC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs2120019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NBDY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs4826508</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLC30A2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs35623192</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rs35235055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOGLIO LAVORO GENEFOOD CONDIZIONI</t>
   </si>
   <si>
     <t xml:space="preserve">Vegano</t>
@@ -1714,7 +1723,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -1798,10 +1807,10 @@
         <v>20</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1810,16 +1819,16 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1828,16 +1837,16 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1846,16 +1855,16 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1863,10 +1872,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -1877,25 +1886,25 @@
         <v>1</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1903,25 +1912,25 @@
         <v>2</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G16" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1929,25 +1938,25 @@
         <v>3</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G17" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="H17" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1955,25 +1964,25 @@
         <v>4</v>
       </c>
       <c r="B18" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="G18" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G18" s="19" t="s">
+      <c r="H18" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1981,25 +1990,25 @@
         <v>5</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D19" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F19" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2007,25 +2016,25 @@
         <v>6</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D20" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2033,25 +2042,25 @@
         <v>7</v>
       </c>
       <c r="B21" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="G21" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>35</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>53</v>
-      </c>
       <c r="H21" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2059,25 +2068,25 @@
         <v>8</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2085,25 +2094,25 @@
         <v>9</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C23" s="24" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I23" s="7"/>
     </row>
@@ -2112,25 +2121,25 @@
         <v>10</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I24" s="7"/>
     </row>
@@ -2139,25 +2148,25 @@
         <v>11</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I25" s="7"/>
     </row>
@@ -2166,25 +2175,25 @@
         <v>12</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I26" s="7"/>
     </row>
@@ -2193,25 +2202,25 @@
         <v>13</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C27" s="24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G27" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="H27" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="H27" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="I27" s="7"/>
     </row>
@@ -2220,25 +2229,25 @@
         <v>14</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D28" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F28" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I28" s="7"/>
     </row>
@@ -2247,25 +2256,25 @@
         <v>15</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C29" s="24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I29" s="7"/>
     </row>
@@ -2274,25 +2283,25 @@
         <v>16</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I30" s="7"/>
     </row>
@@ -2301,25 +2310,25 @@
         <v>17</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I31" s="7"/>
     </row>
@@ -2328,25 +2337,25 @@
         <v>18</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I32" s="7"/>
     </row>
@@ -2355,25 +2364,25 @@
         <v>19</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I33" s="7"/>
     </row>
@@ -2382,25 +2391,25 @@
         <v>20</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I34" s="7"/>
     </row>
@@ -2409,25 +2418,25 @@
         <v>21</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D35" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E35" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E35" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F35" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I35" s="7"/>
     </row>
@@ -2436,25 +2445,25 @@
         <v>22</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I36" s="7"/>
     </row>
@@ -2463,25 +2472,25 @@
         <v>23</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G37" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="H37" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="I37" s="7"/>
     </row>
@@ -2490,25 +2499,25 @@
         <v>24</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D38" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E38" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E38" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F38" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I38" s="7"/>
     </row>
@@ -2517,25 +2526,25 @@
         <v>25</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E39" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G39" s="19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I39" s="7"/>
     </row>
@@ -2544,25 +2553,25 @@
         <v>26</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G40" s="19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I40" s="7"/>
     </row>
@@ -2571,25 +2580,25 @@
         <v>27</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G41" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="H41" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="H41" s="12" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2597,25 +2606,25 @@
         <v>28</v>
       </c>
       <c r="B42" s="30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D42" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E42" s="17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G42" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="H42" s="12" t="s">
         <v>42</v>
-      </c>
-      <c r="H42" s="12" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2623,25 +2632,25 @@
         <v>29</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D43" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E43" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E43" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F43" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2649,51 +2658,51 @@
         <v>30</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D44" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="n">
         <v>31</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D45" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E45" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E45" s="18" t="s">
-        <v>35</v>
-      </c>
       <c r="F45" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -2750,7 +2759,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -2839,7 +2848,7 @@
       <c r="J5" s="37"/>
       <c r="K5" s="38"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E6" s="39" t="s">
         <v>9</v>
       </c>
@@ -2904,10 +2913,10 @@
         <v>19</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H10" s="19"/>
       <c r="I10" s="36"/>
@@ -2916,13 +2925,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="34" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H11" s="36"/>
       <c r="I11" s="37"/>
@@ -2931,13 +2940,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E12" s="34" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H12" s="40"/>
       <c r="I12" s="41"/>
@@ -2946,13 +2955,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E13" s="34" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="4"/>
@@ -2961,10 +2970,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="44" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2972,22 +2981,22 @@
         <v>1</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15" s="46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E15" s="47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H15" s="19"/>
       <c r="I15" s="36"/>
@@ -2999,22 +3008,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D16" s="47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E16" s="46" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="36"/>
@@ -3026,22 +3035,22 @@
         <v>3</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D17" s="46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E17" s="47" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H17" s="19"/>
       <c r="I17" s="36"/>
@@ -3053,22 +3062,22 @@
         <v>4</v>
       </c>
       <c r="B18" s="48" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D18" s="47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E18" s="46" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="36"/>
@@ -3080,22 +3089,22 @@
         <v>5</v>
       </c>
       <c r="B19" s="48" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C19" s="48" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D19" s="47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E19" s="46" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="36"/>
@@ -3107,22 +3116,22 @@
         <v>6</v>
       </c>
       <c r="B20" s="48" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="48" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D20" s="47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E20" s="46" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H20" s="19"/>
       <c r="I20" s="36"/>
@@ -3134,22 +3143,22 @@
         <v>7</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D21" s="47" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E21" s="46" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="36"/>
@@ -3161,22 +3170,22 @@
         <v>8</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D22" s="47" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E22" s="46" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H22" s="19"/>
       <c r="I22" s="36"/>
@@ -3188,22 +3197,22 @@
         <v>9</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D23" s="49" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" s="50" t="s">
+        <v>122</v>
+      </c>
+      <c r="F23" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>120</v>
-      </c>
       <c r="G23" s="12" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="36"/>
@@ -3258,7 +3267,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="52.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="52" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -3359,7 +3368,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>7</v>
+        <v>125</v>
       </c>
       <c r="G5" s="55" t="s">
         <v>8</v>
@@ -3498,10 +3507,10 @@
         <v>19</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H10" s="35"/>
       <c r="I10" s="36"/>
@@ -3520,13 +3529,13 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H11" s="35"/>
       <c r="I11" s="36"/>
@@ -3545,13 +3554,13 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H12" s="35"/>
       <c r="I12" s="36"/>
@@ -3570,13 +3579,13 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H13" s="35"/>
       <c r="I13" s="36"/>
@@ -3594,10 +3603,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -3617,22 +3626,22 @@
         <v>1</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D15" s="58" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H15" s="19"/>
       <c r="I15" s="36"/>
@@ -3650,22 +3659,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C16" s="57" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F16" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="36"/>
@@ -3683,22 +3692,22 @@
         <v>3</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H17" s="19"/>
       <c r="I17" s="36"/>
@@ -3716,22 +3725,22 @@
         <v>4</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="36"/>
@@ -3749,22 +3758,22 @@
         <v>5</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C19" s="60" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="36"/>
@@ -3782,22 +3791,22 @@
         <v>6</v>
       </c>
       <c r="B20" s="61" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C20" s="61" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D20" s="58" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="22" t="s">
-        <v>35</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H20" s="19"/>
       <c r="I20" s="36"/>
@@ -3815,22 +3824,22 @@
         <v>7</v>
       </c>
       <c r="B21" s="57" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C21" s="57" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D21" s="58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="36"/>
@@ -3848,22 +3857,22 @@
         <v>8</v>
       </c>
       <c r="B22" s="57" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C22" s="57" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F22" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>46</v>
       </c>
       <c r="H22" s="19"/>
       <c r="I22" s="36"/>
@@ -3881,22 +3890,22 @@
         <v>9</v>
       </c>
       <c r="B23" s="61" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C23" s="61" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="36"/>
@@ -3914,22 +3923,22 @@
         <v>10</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H24" s="19"/>
       <c r="I24" s="36"/>
@@ -4020,7 +4029,7 @@
   <sheetData>
     <row r="1" s="63" customFormat="true" ht="58.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -4098,7 +4107,7 @@
       <c r="E5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="54"/>
@@ -4106,7 +4115,7 @@
       <c r="I5" s="36"/>
       <c r="J5" s="37"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -4179,7 +4188,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="54"/>
       <c r="H10" s="35"/>
@@ -4192,10 +4201,10 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G11" s="11"/>
       <c r="H11" s="35"/>
@@ -4208,10 +4217,10 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="56"/>
       <c r="H12" s="40"/>
@@ -4224,10 +4233,10 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
@@ -4239,10 +4248,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="53"/>
       <c r="G14" s="4"/>
@@ -4255,19 +4264,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F15" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G15" s="54"/>
       <c r="H15" s="19"/>
@@ -4279,19 +4288,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C16" s="57" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G16" s="54"/>
       <c r="H16" s="19"/>
@@ -4303,19 +4312,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17" s="55" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G17" s="54"/>
       <c r="H17" s="19"/>
@@ -4327,19 +4336,19 @@
         <v>4</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F18" s="55" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G18" s="54"/>
       <c r="H18" s="19"/>
@@ -4351,19 +4360,19 @@
         <v>5</v>
       </c>
       <c r="B19" s="57" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" s="55" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G19" s="54"/>
       <c r="H19" s="19"/>
@@ -4375,19 +4384,19 @@
         <v>6</v>
       </c>
       <c r="B20" s="57" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C20" s="57" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F20" s="55" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="19"/>
@@ -4399,19 +4408,19 @@
         <v>7</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C21" s="60" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F21" s="55" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G21" s="54"/>
       <c r="H21" s="19"/>
@@ -4423,19 +4432,19 @@
         <v>8</v>
       </c>
       <c r="B22" s="61" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C22" s="61" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F22" s="55" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="19"/>
@@ -4447,19 +4456,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D23" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F23" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="19"/>
@@ -4471,19 +4480,19 @@
         <v>10</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D24" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F24" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="19"/>
@@ -4495,19 +4504,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F25" s="55" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G25" s="54"/>
       <c r="H25" s="19"/>
@@ -4519,19 +4528,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="57" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C26" s="57" t="s">
+        <v>163</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" s="55" t="s">
         <v>161</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" s="55" t="s">
-        <v>159</v>
       </c>
       <c r="G26" s="54"/>
       <c r="H26" s="19"/>
@@ -4543,19 +4552,19 @@
         <v>13</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C27" s="57" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F27" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G27" s="54"/>
       <c r="H27" s="19"/>
@@ -4567,19 +4576,19 @@
         <v>14</v>
       </c>
       <c r="B28" s="57" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C28" s="57" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D28" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F28" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G28" s="54"/>
       <c r="H28" s="19"/>
@@ -4591,19 +4600,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="57" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F29" s="55" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G29" s="54"/>
       <c r="H29" s="19"/>
@@ -4615,19 +4624,19 @@
         <v>16</v>
       </c>
       <c r="B30" s="57" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C30" s="57" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F30" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G30" s="54"/>
       <c r="H30" s="19"/>
@@ -4793,7 +4802,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="75" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B1" s="75"/>
       <c r="C1" s="75"/>
@@ -4873,7 +4882,7 @@
       <c r="E5" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="55" t="s">
+      <c r="F5" s="12" t="s">
         <v>7</v>
       </c>
       <c r="G5" s="54"/>
@@ -4881,7 +4890,7 @@
       <c r="I5" s="36"/>
       <c r="J5" s="37"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -4954,7 +4963,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="54"/>
       <c r="H10" s="35"/>
@@ -4967,10 +4976,10 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G11" s="11"/>
       <c r="H11" s="35"/>
@@ -4983,10 +4992,10 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G12" s="56"/>
       <c r="H12" s="77"/>
@@ -4999,10 +5008,10 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
@@ -5014,10 +5023,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="53"/>
       <c r="G14" s="4"/>
@@ -5030,19 +5039,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D15" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F15" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G15" s="54"/>
       <c r="H15" s="19"/>
@@ -5054,19 +5063,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C16" s="57" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D16" s="78" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E16" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G16" s="54"/>
       <c r="H16" s="19"/>
@@ -5078,19 +5087,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F17" s="55" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G17" s="54"/>
       <c r="H17" s="19"/>
@@ -5102,19 +5111,19 @@
         <v>4</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D18" s="78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F18" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G18" s="54"/>
       <c r="H18" s="19"/>
@@ -5126,19 +5135,19 @@
         <v>5</v>
       </c>
       <c r="B19" s="57" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D19" s="78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F19" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G19" s="54"/>
       <c r="H19" s="19"/>
@@ -5150,19 +5159,19 @@
         <v>6</v>
       </c>
       <c r="B20" s="57" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C20" s="57" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D20" s="78" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F20" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="19"/>
@@ -5174,19 +5183,19 @@
         <v>7</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C21" s="60" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D21" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F21" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G21" s="54"/>
       <c r="H21" s="19"/>
@@ -5198,19 +5207,19 @@
         <v>8</v>
       </c>
       <c r="B22" s="61" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C22" s="61" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D22" s="78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F22" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="19"/>
@@ -5222,19 +5231,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D23" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="E23" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F23" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="19"/>
@@ -5246,19 +5255,19 @@
         <v>10</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D24" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F24" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="19"/>
@@ -5270,19 +5279,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D25" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="E25" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F25" s="55" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G25" s="54"/>
       <c r="H25" s="19"/>
@@ -5294,19 +5303,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="57" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C26" s="57" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D26" s="78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F26" s="55" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G26" s="54"/>
       <c r="H26" s="19"/>
@@ -5318,19 +5327,19 @@
         <v>13</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C27" s="57" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D27" s="78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F27" s="55" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G27" s="54"/>
       <c r="H27" s="19"/>
@@ -5342,19 +5351,19 @@
         <v>14</v>
       </c>
       <c r="B28" s="57" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C28" s="57" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D28" s="78" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F28" s="55" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G28" s="54"/>
       <c r="H28" s="19"/>
@@ -5366,19 +5375,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="57" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D29" s="78" t="s">
+        <v>37</v>
+      </c>
+      <c r="E29" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E29" s="28" t="s">
-        <v>35</v>
-      </c>
       <c r="F29" s="55" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G29" s="54"/>
       <c r="H29" s="19"/>
@@ -5442,7 +5451,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="43.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -5527,7 +5536,7 @@
       <c r="I5" s="36"/>
       <c r="J5" s="37"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -5597,10 +5606,10 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G10" s="54"/>
       <c r="H10" s="19"/>
@@ -5613,10 +5622,10 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G11" s="54"/>
       <c r="H11" s="19"/>
@@ -5629,10 +5638,10 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G12" s="56"/>
       <c r="H12" s="40"/>
@@ -5645,10 +5654,10 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
@@ -5660,10 +5669,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -5676,19 +5685,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="80" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C15" s="80" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D15" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="E15" s="58" t="s">
-        <v>35</v>
-      </c>
       <c r="F15" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G15" s="54"/>
       <c r="H15" s="19"/>
@@ -5700,19 +5709,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="80" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C16" s="80" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E16" s="58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G16" s="54"/>
       <c r="H16" s="19"/>
@@ -5724,19 +5733,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D17" s="58" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E17" s="81" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G17" s="54"/>
       <c r="H17" s="19"/>
@@ -5748,19 +5757,19 @@
         <v>4</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E18" s="58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G18" s="54"/>
       <c r="H18" s="19"/>
@@ -5772,19 +5781,19 @@
         <v>5</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D19" s="58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E19" s="81" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G19" s="54"/>
       <c r="H19" s="19"/>
@@ -5796,19 +5805,19 @@
         <v>6</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D20" s="58" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="81" t="s">
         <v>36</v>
       </c>
-      <c r="E20" s="81" t="s">
-        <v>35</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="19"/>
@@ -5820,19 +5829,19 @@
         <v>7</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D21" s="58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E21" s="81" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G21" s="54"/>
       <c r="H21" s="19"/>
@@ -5844,19 +5853,19 @@
         <v>8</v>
       </c>
       <c r="B22" s="80" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C22" s="80" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D22" s="58" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E22" s="81" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="19"/>
@@ -5868,19 +5877,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="80" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C23" s="80" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D23" s="58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E23" s="81" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="19"/>
@@ -5892,19 +5901,19 @@
         <v>10</v>
       </c>
       <c r="B24" s="80" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C24" s="80" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D24" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="E24" s="58" t="s">
-        <v>35</v>
-      </c>
       <c r="F24" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="19"/>
@@ -5916,19 +5925,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="80" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C25" s="80" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D25" s="58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E25" s="81" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G25" s="54"/>
       <c r="H25" s="19"/>
@@ -5940,19 +5949,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="80" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C26" s="80" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D26" s="58" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E26" s="81" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G26" s="54"/>
       <c r="H26" s="19"/>
@@ -5964,19 +5973,19 @@
         <v>13</v>
       </c>
       <c r="B27" s="80" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C27" s="80" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D27" s="81" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E27" s="58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G27" s="54"/>
       <c r="H27" s="19"/>
@@ -5988,19 +5997,19 @@
         <v>14</v>
       </c>
       <c r="B28" s="80" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C28" s="80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D28" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" s="58" t="s">
         <v>36</v>
       </c>
-      <c r="E28" s="58" t="s">
-        <v>35</v>
-      </c>
       <c r="F28" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G28" s="54"/>
       <c r="H28" s="19"/>
@@ -6012,19 +6021,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="80" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C29" s="80" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D29" s="58" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G29" s="54"/>
       <c r="H29" s="19"/>
@@ -6036,19 +6045,19 @@
         <v>16</v>
       </c>
       <c r="B30" s="80" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C30" s="80" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E30" s="58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G30" s="54"/>
       <c r="H30" s="19"/>
@@ -6060,19 +6069,19 @@
         <v>17</v>
       </c>
       <c r="B31" s="80" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C31" s="80" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D31" s="58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G31" s="54"/>
       <c r="H31" s="19"/>
@@ -6208,7 +6217,7 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="51" width="17.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="51" width="17.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="36.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="33.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="23.48"/>
@@ -6216,7 +6225,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6285,7 +6294,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>6</v>
+        <v>224</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>7</v>
@@ -6294,7 +6303,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -6375,13 +6384,13 @@
         <v>19</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6390,16 +6399,16 @@
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6408,16 +6417,16 @@
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6426,16 +6435,16 @@
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="51.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6444,13 +6453,13 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="88" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F14" s="89" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="G14" s="89" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="H14" s="89"/>
     </row>

</xml_diff>

<commit_message>
Braincare as new commitent; added app instructions at the end of reports
</commit_message>
<xml_diff>
--- a/static/esempio_paziente_completo_filled.xlsx
+++ b/static/esempio_paziente_completo_filled.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="230">
   <si>
     <t xml:space="preserve">FOGLIO LAVORO GENEFOOD BASE</t>
   </si>
@@ -123,6 +123,9 @@
   </si>
   <si>
     <t xml:space="preserve">COMMITTENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Braincare</t>
   </si>
   <si>
     <t xml:space="preserve">Genessere</t>
@@ -1861,10 +1864,10 @@
         <v>30</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1872,10 +1875,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -1886,25 +1889,25 @@
         <v>1</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1912,25 +1915,25 @@
         <v>2</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G16" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1938,25 +1941,25 @@
         <v>3</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G17" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="H17" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1964,25 +1967,25 @@
         <v>4</v>
       </c>
       <c r="B18" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" s="19" t="s">
+      <c r="H18" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1990,25 +1993,25 @@
         <v>5</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D19" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E19" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F19" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H19" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2016,25 +2019,25 @@
         <v>6</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D20" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2042,25 +2045,25 @@
         <v>7</v>
       </c>
       <c r="B21" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="G21" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>54</v>
-      </c>
       <c r="H21" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2068,25 +2071,25 @@
         <v>8</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H22" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2094,25 +2097,25 @@
         <v>9</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C23" s="24" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H23" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I23" s="7"/>
     </row>
@@ -2121,25 +2124,25 @@
         <v>10</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I24" s="7"/>
     </row>
@@ -2148,25 +2151,25 @@
         <v>11</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I25" s="7"/>
     </row>
@@ -2175,25 +2178,25 @@
         <v>12</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I26" s="7"/>
     </row>
@@ -2202,25 +2205,25 @@
         <v>13</v>
       </c>
       <c r="B27" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C27" s="24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G27" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="H27" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="H27" s="12" t="s">
-        <v>47</v>
       </c>
       <c r="I27" s="7"/>
     </row>
@@ -2229,25 +2232,25 @@
         <v>14</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C28" s="16" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D28" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F28" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G28" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I28" s="7"/>
     </row>
@@ -2256,25 +2259,25 @@
         <v>15</v>
       </c>
       <c r="B29" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C29" s="24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G29" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I29" s="7"/>
     </row>
@@ -2283,25 +2286,25 @@
         <v>16</v>
       </c>
       <c r="B30" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E30" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G30" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I30" s="7"/>
     </row>
@@ -2310,25 +2313,25 @@
         <v>17</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C31" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I31" s="7"/>
     </row>
@@ -2337,25 +2340,25 @@
         <v>18</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C32" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I32" s="7"/>
     </row>
@@ -2364,25 +2367,25 @@
         <v>19</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G33" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I33" s="7"/>
     </row>
@@ -2391,25 +2394,25 @@
         <v>20</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G34" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I34" s="7"/>
     </row>
@@ -2418,25 +2421,25 @@
         <v>21</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D35" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E35" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E35" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F35" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I35" s="7"/>
     </row>
@@ -2445,25 +2448,25 @@
         <v>22</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H36" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I36" s="7"/>
     </row>
@@ -2472,25 +2475,25 @@
         <v>23</v>
       </c>
       <c r="B37" s="25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G37" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="H37" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>47</v>
       </c>
       <c r="I37" s="7"/>
     </row>
@@ -2499,25 +2502,25 @@
         <v>24</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C38" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D38" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E38" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F38" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G38" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I38" s="7"/>
     </row>
@@ -2526,25 +2529,25 @@
         <v>25</v>
       </c>
       <c r="B39" s="27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C39" s="25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E39" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G39" s="19" t="s">
         <v>24</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I39" s="7"/>
     </row>
@@ -2553,25 +2556,25 @@
         <v>26</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C40" s="29" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D40" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G40" s="19" t="s">
         <v>24</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I40" s="7"/>
     </row>
@@ -2580,25 +2583,25 @@
         <v>27</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C41" s="16" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D41" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E41" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G41" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="H41" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="H41" s="12" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2606,25 +2609,25 @@
         <v>28</v>
       </c>
       <c r="B42" s="30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C42" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D42" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E42" s="17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G42" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="H42" s="12" t="s">
         <v>43</v>
-      </c>
-      <c r="H42" s="12" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2632,25 +2635,25 @@
         <v>29</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D43" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E43" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E43" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F43" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G43" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H43" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2658,25 +2661,25 @@
         <v>30</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D44" s="18" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E44" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G44" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H44" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2684,25 +2687,25 @@
         <v>31</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D45" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E45" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E45" s="18" t="s">
-        <v>36</v>
-      </c>
       <c r="F45" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G45" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H45" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2711,9 +2714,13 @@
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="F2:H2"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F13" type="list">
-      <formula1>"Altamedica,Genessere"</formula1>
+      <formula1>"Altamedica,Genessere,Braincare"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G13" type="list">
+      <formula1>"Altamedica,Genessere,Braincare"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2759,7 +2766,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="45.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -2958,10 +2965,10 @@
         <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H13" s="14"/>
       <c r="I13" s="4"/>
@@ -2970,10 +2977,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="44" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="45" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2981,22 +2988,22 @@
         <v>1</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D15" s="46" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E15" s="47" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H15" s="19"/>
       <c r="I15" s="36"/>
@@ -3008,22 +3015,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D16" s="47" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" s="46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G16" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="36"/>
@@ -3035,22 +3042,22 @@
         <v>3</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D17" s="46" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="47" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H17" s="19"/>
       <c r="I17" s="36"/>
@@ -3062,22 +3069,22 @@
         <v>4</v>
       </c>
       <c r="B18" s="48" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" s="47" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E18" s="46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="36"/>
@@ -3089,22 +3096,22 @@
         <v>5</v>
       </c>
       <c r="B19" s="48" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="48" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D19" s="47" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" s="46" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="36"/>
@@ -3116,22 +3123,22 @@
         <v>6</v>
       </c>
       <c r="B20" s="48" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C20" s="48" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D20" s="47" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E20" s="46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H20" s="19"/>
       <c r="I20" s="36"/>
@@ -3143,22 +3150,22 @@
         <v>7</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D21" s="47" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E21" s="46" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="36"/>
@@ -3170,22 +3177,22 @@
         <v>8</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D22" s="47" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E22" s="46" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H22" s="19"/>
       <c r="I22" s="36"/>
@@ -3197,22 +3204,22 @@
         <v>9</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D23" s="49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E23" s="50" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="F23" s="12" t="s">
-        <v>121</v>
-      </c>
       <c r="G23" s="12" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="36"/>
@@ -3229,7 +3236,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F13" type="list">
-      <formula1>"Altamedica,Genessere"</formula1>
+      <formula1>"Altamedica,Genessere,Braincare"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3267,7 +3274,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="52.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="52" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B1" s="52"/>
       <c r="C1" s="52"/>
@@ -3368,7 +3375,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G5" s="55" t="s">
         <v>8</v>
@@ -3582,10 +3589,10 @@
         <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H13" s="35"/>
       <c r="I13" s="36"/>
@@ -3603,10 +3610,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -3626,22 +3633,22 @@
         <v>1</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D15" s="58" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H15" s="19"/>
       <c r="I15" s="36"/>
@@ -3659,22 +3666,22 @@
         <v>2</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C16" s="57" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D16" s="58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F16" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>47</v>
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="36"/>
@@ -3692,22 +3699,22 @@
         <v>3</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G17" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H17" s="19"/>
       <c r="I17" s="36"/>
@@ -3725,22 +3732,22 @@
         <v>4</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D18" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G18" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="36"/>
@@ -3758,22 +3765,22 @@
         <v>5</v>
       </c>
       <c r="B19" s="60" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C19" s="60" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="36"/>
@@ -3791,22 +3798,22 @@
         <v>6</v>
       </c>
       <c r="B20" s="61" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C20" s="61" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D20" s="58" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="22" t="s">
-        <v>36</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H20" s="19"/>
       <c r="I20" s="36"/>
@@ -3824,22 +3831,22 @@
         <v>7</v>
       </c>
       <c r="B21" s="57" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C21" s="57" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D21" s="58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G21" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="36"/>
@@ -3857,22 +3864,22 @@
         <v>8</v>
       </c>
       <c r="B22" s="57" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C22" s="57" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F22" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>47</v>
       </c>
       <c r="H22" s="19"/>
       <c r="I22" s="36"/>
@@ -3890,22 +3897,22 @@
         <v>9</v>
       </c>
       <c r="B23" s="61" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C23" s="61" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="36"/>
@@ -3923,22 +3930,22 @@
         <v>10</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E24" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H24" s="19"/>
       <c r="I24" s="36"/>
@@ -3984,7 +3991,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F13" type="list">
-      <formula1>"Altamedica,Genessere"</formula1>
+      <formula1>"Altamedica,Genessere,Braincare"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4029,7 +4036,7 @@
   <sheetData>
     <row r="1" s="63" customFormat="true" ht="58.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="62" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B1" s="62"/>
       <c r="C1" s="62"/>
@@ -4248,10 +4255,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F14" s="53"/>
       <c r="G14" s="4"/>
@@ -4264,19 +4271,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E15" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F15" s="55" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G15" s="54"/>
       <c r="H15" s="19"/>
@@ -4288,19 +4295,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C16" s="57" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D16" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G16" s="54"/>
       <c r="H16" s="19"/>
@@ -4312,19 +4319,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D17" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F17" s="55" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G17" s="54"/>
       <c r="H17" s="19"/>
@@ -4336,19 +4343,19 @@
         <v>4</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F18" s="55" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G18" s="54"/>
       <c r="H18" s="19"/>
@@ -4360,19 +4367,19 @@
         <v>5</v>
       </c>
       <c r="B19" s="57" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D19" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F19" s="55" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G19" s="54"/>
       <c r="H19" s="19"/>
@@ -4384,19 +4391,19 @@
         <v>6</v>
       </c>
       <c r="B20" s="57" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C20" s="57" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F20" s="55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="19"/>
@@ -4408,19 +4415,19 @@
         <v>7</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C21" s="60" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D21" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F21" s="55" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G21" s="54"/>
       <c r="H21" s="19"/>
@@ -4432,19 +4439,19 @@
         <v>8</v>
       </c>
       <c r="B22" s="61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C22" s="61" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F22" s="55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="19"/>
@@ -4456,19 +4463,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D23" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F23" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="19"/>
@@ -4480,19 +4487,19 @@
         <v>10</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D24" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E24" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F24" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="19"/>
@@ -4504,19 +4511,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E25" s="28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F25" s="55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G25" s="54"/>
       <c r="H25" s="19"/>
@@ -4528,19 +4535,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="57" t="s">
+        <v>163</v>
+      </c>
+      <c r="C26" s="57" t="s">
+        <v>164</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="55" t="s">
         <v>162</v>
-      </c>
-      <c r="C26" s="57" t="s">
-        <v>163</v>
-      </c>
-      <c r="D26" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="F26" s="55" t="s">
-        <v>161</v>
       </c>
       <c r="G26" s="54"/>
       <c r="H26" s="19"/>
@@ -4552,19 +4559,19 @@
         <v>13</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C27" s="57" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F27" s="55" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G27" s="54"/>
       <c r="H27" s="19"/>
@@ -4576,19 +4583,19 @@
         <v>14</v>
       </c>
       <c r="B28" s="57" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C28" s="57" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D28" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F28" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G28" s="54"/>
       <c r="H28" s="19"/>
@@ -4600,19 +4607,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="57" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D29" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F29" s="55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G29" s="54"/>
       <c r="H29" s="19"/>
@@ -4624,19 +4631,19 @@
         <v>16</v>
       </c>
       <c r="B30" s="57" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C30" s="57" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D30" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F30" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G30" s="54"/>
       <c r="H30" s="19"/>
@@ -4802,7 +4809,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="75" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B1" s="75"/>
       <c r="C1" s="75"/>
@@ -5023,10 +5030,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F14" s="53"/>
       <c r="G14" s="4"/>
@@ -5039,19 +5046,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="57" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C15" s="57" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D15" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F15" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G15" s="54"/>
       <c r="H15" s="19"/>
@@ -5063,19 +5070,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="57" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C16" s="57" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D16" s="78" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E16" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F16" s="55" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G16" s="54"/>
       <c r="H16" s="19"/>
@@ -5087,19 +5094,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="57" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C17" s="57" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D17" s="79" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F17" s="55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G17" s="54"/>
       <c r="H17" s="19"/>
@@ -5111,19 +5118,19 @@
         <v>4</v>
       </c>
       <c r="B18" s="57" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D18" s="78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E18" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F18" s="55" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G18" s="54"/>
       <c r="H18" s="19"/>
@@ -5135,19 +5142,19 @@
         <v>5</v>
       </c>
       <c r="B19" s="57" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C19" s="57" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D19" s="78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E19" s="28" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G19" s="54"/>
       <c r="H19" s="19"/>
@@ -5159,19 +5166,19 @@
         <v>6</v>
       </c>
       <c r="B20" s="57" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C20" s="57" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D20" s="78" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E20" s="28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F20" s="55" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="19"/>
@@ -5183,19 +5190,19 @@
         <v>7</v>
       </c>
       <c r="B21" s="60" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C21" s="60" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D21" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F21" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G21" s="54"/>
       <c r="H21" s="19"/>
@@ -5207,19 +5214,19 @@
         <v>8</v>
       </c>
       <c r="B22" s="61" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C22" s="61" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D22" s="78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E22" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F22" s="55" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="19"/>
@@ -5231,19 +5238,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="57" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D23" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="E23" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F23" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="19"/>
@@ -5255,19 +5262,19 @@
         <v>10</v>
       </c>
       <c r="B24" s="57" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D24" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E24" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F24" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="19"/>
@@ -5279,19 +5286,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="57" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D25" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E25" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F25" s="55" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G25" s="54"/>
       <c r="H25" s="19"/>
@@ -5303,19 +5310,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="57" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C26" s="57" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D26" s="78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E26" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F26" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G26" s="54"/>
       <c r="H26" s="19"/>
@@ -5327,19 +5334,19 @@
         <v>13</v>
       </c>
       <c r="B27" s="57" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C27" s="57" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D27" s="78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E27" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F27" s="55" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G27" s="54"/>
       <c r="H27" s="19"/>
@@ -5351,19 +5358,19 @@
         <v>14</v>
       </c>
       <c r="B28" s="57" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C28" s="57" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D28" s="78" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E28" s="28" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F28" s="55" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G28" s="54"/>
       <c r="H28" s="19"/>
@@ -5375,19 +5382,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="57" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D29" s="78" t="s">
+        <v>38</v>
+      </c>
+      <c r="E29" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="E29" s="28" t="s">
-        <v>36</v>
-      </c>
       <c r="F29" s="55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G29" s="54"/>
       <c r="H29" s="19"/>
@@ -5451,7 +5458,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="43.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -5606,7 +5613,7 @@
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="10" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F10" s="11" t="s">
         <v>22</v>
@@ -5657,7 +5664,7 @@
         <v>29</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G13" s="14"/>
       <c r="H13" s="14"/>
@@ -5669,10 +5676,10 @@
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
       <c r="D14" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>
@@ -5685,19 +5692,19 @@
         <v>1</v>
       </c>
       <c r="B15" s="80" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C15" s="80" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D15" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="58" t="s">
-        <v>36</v>
-      </c>
       <c r="F15" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G15" s="54"/>
       <c r="H15" s="19"/>
@@ -5709,19 +5716,19 @@
         <v>2</v>
       </c>
       <c r="B16" s="80" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C16" s="80" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E16" s="58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G16" s="54"/>
       <c r="H16" s="19"/>
@@ -5733,19 +5740,19 @@
         <v>3</v>
       </c>
       <c r="B17" s="80" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C17" s="80" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D17" s="58" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E17" s="81" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G17" s="54"/>
       <c r="H17" s="19"/>
@@ -5757,19 +5764,19 @@
         <v>4</v>
       </c>
       <c r="B18" s="80" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C18" s="80" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E18" s="58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G18" s="54"/>
       <c r="H18" s="19"/>
@@ -5781,19 +5788,19 @@
         <v>5</v>
       </c>
       <c r="B19" s="80" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C19" s="80" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D19" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E19" s="81" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G19" s="54"/>
       <c r="H19" s="19"/>
@@ -5805,19 +5812,19 @@
         <v>6</v>
       </c>
       <c r="B20" s="80" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C20" s="80" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D20" s="58" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" s="81" t="s">
         <v>37</v>
       </c>
-      <c r="E20" s="81" t="s">
-        <v>36</v>
-      </c>
       <c r="F20" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G20" s="54"/>
       <c r="H20" s="19"/>
@@ -5829,19 +5836,19 @@
         <v>7</v>
       </c>
       <c r="B21" s="80" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C21" s="80" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D21" s="58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E21" s="81" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G21" s="54"/>
       <c r="H21" s="19"/>
@@ -5853,19 +5860,19 @@
         <v>8</v>
       </c>
       <c r="B22" s="80" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C22" s="80" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D22" s="58" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E22" s="81" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G22" s="54"/>
       <c r="H22" s="19"/>
@@ -5877,19 +5884,19 @@
         <v>9</v>
       </c>
       <c r="B23" s="80" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C23" s="80" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D23" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E23" s="81" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G23" s="54"/>
       <c r="H23" s="19"/>
@@ -5901,19 +5908,19 @@
         <v>10</v>
       </c>
       <c r="B24" s="80" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C24" s="80" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D24" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="E24" s="58" t="s">
-        <v>36</v>
-      </c>
       <c r="F24" s="12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G24" s="54"/>
       <c r="H24" s="19"/>
@@ -5925,19 +5932,19 @@
         <v>11</v>
       </c>
       <c r="B25" s="80" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C25" s="80" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D25" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E25" s="81" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G25" s="54"/>
       <c r="H25" s="19"/>
@@ -5949,19 +5956,19 @@
         <v>12</v>
       </c>
       <c r="B26" s="80" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C26" s="80" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D26" s="58" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E26" s="81" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G26" s="54"/>
       <c r="H26" s="19"/>
@@ -5973,19 +5980,19 @@
         <v>13</v>
       </c>
       <c r="B27" s="80" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C27" s="80" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D27" s="81" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E27" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G27" s="54"/>
       <c r="H27" s="19"/>
@@ -5997,19 +6004,19 @@
         <v>14</v>
       </c>
       <c r="B28" s="80" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C28" s="80" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D28" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E28" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="E28" s="58" t="s">
-        <v>36</v>
-      </c>
       <c r="F28" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G28" s="54"/>
       <c r="H28" s="19"/>
@@ -6021,19 +6028,19 @@
         <v>15</v>
       </c>
       <c r="B29" s="80" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C29" s="80" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D29" s="58" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G29" s="54"/>
       <c r="H29" s="19"/>
@@ -6045,19 +6052,19 @@
         <v>16</v>
       </c>
       <c r="B30" s="80" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C30" s="80" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E30" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G30" s="54"/>
       <c r="H30" s="19"/>
@@ -6069,19 +6076,19 @@
         <v>17</v>
       </c>
       <c r="B31" s="80" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C31" s="80" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D31" s="58" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G31" s="54"/>
       <c r="H31" s="19"/>
@@ -6225,7 +6232,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -6294,7 +6301,7 @@
         <v>5</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>7</v>
@@ -6402,7 +6409,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>24</v>
@@ -6441,10 +6448,10 @@
         <v>30</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="51.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6453,13 +6460,13 @@
       <c r="C14" s="4"/>
       <c r="D14" s="4"/>
       <c r="E14" s="88" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F14" s="89" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G14" s="89" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H14" s="89"/>
     </row>
@@ -6471,7 +6478,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F13" type="list">
-      <formula1>"Altamedica,Genessere"</formula1>
+      <formula1>"Altamedica,Genessere,Braincare"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
restored nichel in Junior_intoll
</commit_message>
<xml_diff>
--- a/static/esempio_paziente_completo_filled.xlsx
+++ b/static/esempio_paziente_completo_filled.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t xml:space="preserve">FOGLIO LAVORO GENEFOOD CONDIZIONI</t>
   </si>
@@ -109,10 +109,13 @@
     <t xml:space="preserve">COMMITTENTE</t>
   </si>
   <si>
+    <t xml:space="preserve">IkonFiumicino</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genessere</t>
+  </si>
+  <si>
     <t xml:space="preserve">Altamedica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Genessere</t>
   </si>
   <si>
     <t xml:space="preserve">CONDIZIONI</t>
@@ -747,35 +750,35 @@
         <v>30</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" s="26" customFormat="true" ht="51.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" s="26" customFormat="true" ht="24.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="27" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="29" t="s">
         <v>37</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -784,10 +787,6 @@
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B13" type="list">
-      <formula1>"Altamedica,Genessere,Braincare"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B15" type="list">
       <formula1>"Normale,DQ2.5 \ DQ2.5,DQ2.5 \ DQ2.2,DQ2.5 (cis),DQ2.5 (trans),DQ2.2 \ DQ2.2,DQ2.2 \ DQX,DQ8 \ DQ8,DQ8 \ DQX,DQ2.5 \ DQX,DQ2.5 \ DQ8,DQ7 \ DQX,DQ7 \ DQ7,DQ7 \ DQ2.2,DQ7 \ DQ8"</formula1>
       <formula2>0</formula2>
@@ -798,6 +797,10 @@
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D15" type="list">
       <formula1>"Normale,DQ2.5 \ DQ2.5,DQ2.5 \ DQ2.2,DQ2.5 (cis),DQ2.5 (trans),DQ2.2 \ DQ2.2,DQ2.2 \ DQX,DQ8 \ DQ8,DQ8 \ DQX,DQ2.5 \ DQX,DQ2.5 \ DQ8,DQ7 \ DQX,DQ7 \ DQ7,DQ7 \ DQ2.2,DQ7 \ DQ8"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B13" type="list">
+      <formula1>"Altamedica,Genessere,Braincare,Longevia,IkonFiumicino,IkonAcilia,IkonCasalPalocco"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>